<commit_message>
fix copy-paste error for blade cm
</commit_message>
<xml_diff>
--- a/Documentation/IEA-15-240-RWT_tabular.xlsx
+++ b/Documentation/IEA-15-240-RWT_tabular.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gbarter/devel/IEA-15-240-RWT/Documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{126B7BE3-3AFE-C946-B584-E06D5408FAB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56B8FCBE-3DEE-7548-9339-C2710B655D08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17020" yWindow="500" windowWidth="33600" windowHeight="19360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4800" yWindow="620" windowWidth="33600" windowHeight="19360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
@@ -1009,7 +1009,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="2"/>
@@ -1017,7 +1017,6 @@
     <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="1" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Heading 1" xfId="2" builtinId="16"/>
@@ -18151,7 +18150,7 @@
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1100-000000000000}">
-  <dimension ref="A1:Q24"/>
+  <dimension ref="A1:Q26"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13.83203125" bestFit="1" customWidth="1"/>
@@ -18228,52 +18227,52 @@
       <c r="A3" t="s">
         <v>264</v>
       </c>
-      <c r="B3" s="6">
+      <c r="B3">
         <v>48092.001786537301</v>
       </c>
-      <c r="C3" s="5">
+      <c r="C3">
         <v>-7.0885261800196808</v>
       </c>
-      <c r="D3" s="5">
-        <v>0</v>
-      </c>
-      <c r="E3" s="5">
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3">
         <v>5.094493537559762</v>
       </c>
-      <c r="F3" s="6">
+      <c r="F3">
         <v>59002.874691857964</v>
       </c>
-      <c r="G3" s="6">
+      <c r="G3">
         <v>29771.954855978249</v>
       </c>
-      <c r="H3" s="6">
+      <c r="H3">
         <v>29771.954855978249</v>
       </c>
-      <c r="I3" s="6">
-        <v>0</v>
-      </c>
-      <c r="J3" s="6">
-        <v>0</v>
-      </c>
-      <c r="K3" s="6">
-        <v>0</v>
-      </c>
-      <c r="L3" s="6">
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3">
+        <v>0</v>
+      </c>
+      <c r="L3">
         <v>1306856.7851224421</v>
       </c>
-      <c r="M3" s="6">
+      <c r="M3">
         <v>3694433.844065466</v>
       </c>
-      <c r="N3" s="6">
+      <c r="N3">
         <v>2446579.9336348828</v>
       </c>
-      <c r="O3" s="6">
-        <v>0</v>
-      </c>
-      <c r="P3" s="6">
+      <c r="O3">
+        <v>0</v>
+      </c>
+      <c r="P3">
         <v>1733681.3241244019</v>
       </c>
-      <c r="Q3" s="6">
+      <c r="Q3">
         <v>0</v>
       </c>
     </row>
@@ -18281,52 +18280,52 @@
       <c r="A4" t="s">
         <v>265</v>
       </c>
-      <c r="B4" s="6">
+      <c r="B4">
         <v>13479.28387693245</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C4">
         <v>-5.8950999055777533</v>
       </c>
-      <c r="D4" s="5">
-        <v>0</v>
-      </c>
-      <c r="E4" s="5">
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
         <v>4.9690593816385773</v>
       </c>
-      <c r="F4" s="6">
+      <c r="F4">
         <v>16537.3964065115</v>
       </c>
-      <c r="G4" s="6">
+      <c r="G4">
         <v>8344.5191750634949</v>
       </c>
-      <c r="H4" s="6">
+      <c r="H4">
         <v>8344.5191750634949</v>
       </c>
-      <c r="I4" s="6">
-        <v>0</v>
-      </c>
-      <c r="J4" s="6">
-        <v>0</v>
-      </c>
-      <c r="K4" s="6">
-        <v>0</v>
-      </c>
-      <c r="L4" s="6">
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4">
+        <v>0</v>
+      </c>
+      <c r="L4">
         <v>349272.30654858239</v>
       </c>
-      <c r="M4" s="6">
+      <c r="M4">
         <v>809603.75452328555</v>
       </c>
-      <c r="N4" s="6">
+      <c r="N4">
         <v>476868.84438121459</v>
       </c>
-      <c r="O4" s="6">
-        <v>0</v>
-      </c>
-      <c r="P4" s="6">
+      <c r="O4">
+        <v>0</v>
+      </c>
+      <c r="P4">
         <v>393998.33316090098</v>
       </c>
-      <c r="Q4" s="6">
+      <c r="Q4">
         <v>0</v>
       </c>
     </row>
@@ -18334,52 +18333,52 @@
       <c r="A5" t="s">
         <v>266</v>
       </c>
-      <c r="B5" s="6">
+      <c r="B5">
         <v>15734.038486973781</v>
       </c>
-      <c r="C5" s="5">
+      <c r="C5">
         <v>-6.9890739904828534</v>
       </c>
-      <c r="D5" s="5">
-        <v>0</v>
-      </c>
-      <c r="E5" s="5">
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
         <v>5.0840406912329961</v>
       </c>
-      <c r="F5" s="6">
+      <c r="F5">
         <v>33120.151015079799</v>
       </c>
-      <c r="G5" s="6">
+      <c r="G5">
         <v>22906.137697285991</v>
       </c>
-      <c r="H5" s="6">
+      <c r="H5">
         <v>22906.137697285991</v>
       </c>
-      <c r="I5" s="6">
-        <v>0</v>
-      </c>
-      <c r="J5" s="6">
-        <v>0</v>
-      </c>
-      <c r="K5" s="6">
-        <v>0</v>
-      </c>
-      <c r="L5" s="6">
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
+      <c r="K5">
+        <v>0</v>
+      </c>
+      <c r="L5">
         <v>439693.63450568088</v>
       </c>
-      <c r="M5" s="6">
+      <c r="M5">
         <v>1198154.2421317161</v>
       </c>
-      <c r="N5" s="6">
+      <c r="N5">
         <v>791580.75864111481</v>
       </c>
-      <c r="O5" s="6">
-        <v>0</v>
-      </c>
-      <c r="P5" s="6">
+      <c r="O5">
+        <v>0</v>
+      </c>
+      <c r="P5">
         <v>558011.63821907982</v>
       </c>
-      <c r="Q5" s="6">
+      <c r="Q5">
         <v>0</v>
       </c>
     </row>
@@ -18387,52 +18386,52 @@
       <c r="A6" t="s">
         <v>267</v>
       </c>
-      <c r="B6" s="6">
-        <v>0</v>
-      </c>
-      <c r="C6" s="5">
+      <c r="B6">
+        <v>0</v>
+      </c>
+      <c r="C6">
         <v>-5.0000301997463072</v>
       </c>
-      <c r="D6" s="5">
-        <v>0</v>
-      </c>
-      <c r="E6" s="5">
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6">
         <v>4.8749837646976886</v>
       </c>
-      <c r="F6" s="6">
-        <v>0</v>
-      </c>
-      <c r="G6" s="6">
-        <v>0</v>
-      </c>
-      <c r="H6" s="6">
-        <v>0</v>
-      </c>
-      <c r="I6" s="6">
-        <v>0</v>
-      </c>
-      <c r="J6" s="6">
-        <v>0</v>
-      </c>
-      <c r="K6" s="6">
-        <v>0</v>
-      </c>
-      <c r="L6" s="6">
-        <v>0</v>
-      </c>
-      <c r="M6" s="6">
-        <v>0</v>
-      </c>
-      <c r="N6" s="6">
-        <v>0</v>
-      </c>
-      <c r="O6" s="6">
-        <v>0</v>
-      </c>
-      <c r="P6" s="6">
-        <v>0</v>
-      </c>
-      <c r="Q6" s="6">
+      <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
+      <c r="K6">
+        <v>0</v>
+      </c>
+      <c r="L6">
+        <v>0</v>
+      </c>
+      <c r="M6">
+        <v>0</v>
+      </c>
+      <c r="N6">
+        <v>0</v>
+      </c>
+      <c r="O6">
+        <v>0</v>
+      </c>
+      <c r="P6">
+        <v>0</v>
+      </c>
+      <c r="Q6">
         <v>0</v>
       </c>
     </row>
@@ -18440,52 +18439,52 @@
       <c r="A7" t="s">
         <v>268</v>
       </c>
-      <c r="B7" s="6">
-        <v>24290.364248076799</v>
-      </c>
-      <c r="C7" s="5">
+      <c r="B7">
+        <v>22961.01507170952</v>
+      </c>
+      <c r="C7">
         <v>-7.585787127703818</v>
       </c>
-      <c r="D7" s="5">
-        <v>0</v>
-      </c>
-      <c r="E7" s="5">
+      <c r="D7">
+        <v>0</v>
+      </c>
+      <c r="E7">
         <v>5.1467577691935888</v>
       </c>
-      <c r="F7" s="6">
-        <v>17686.462299954401</v>
-      </c>
-      <c r="G7" s="6">
-        <v>8843.2311499772022</v>
-      </c>
-      <c r="H7" s="6">
-        <v>8843.2311499772022</v>
-      </c>
-      <c r="I7" s="6">
-        <v>0</v>
-      </c>
-      <c r="J7" s="6">
-        <v>0</v>
-      </c>
-      <c r="K7" s="6">
-        <v>0</v>
-      </c>
-      <c r="L7" s="6">
-        <v>661020.10433958611</v>
-      </c>
-      <c r="M7" s="6">
-        <v>2050042.257015147</v>
-      </c>
-      <c r="N7" s="6">
-        <v>1406708.6149755151</v>
-      </c>
-      <c r="O7" s="6">
-        <v>0</v>
-      </c>
-      <c r="P7" s="6">
-        <v>947430.16808027821</v>
-      </c>
-      <c r="Q7" s="6">
+      <c r="F7">
+        <v>16718.527696291269</v>
+      </c>
+      <c r="G7">
+        <v>8359.2638481456361</v>
+      </c>
+      <c r="H7">
+        <v>8359.2638481456361</v>
+      </c>
+      <c r="I7">
+        <v>0</v>
+      </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
+      <c r="K7">
+        <v>0</v>
+      </c>
+      <c r="L7">
+        <v>624844.17374045495</v>
+      </c>
+      <c r="M7">
+        <v>1937848.715656582</v>
+      </c>
+      <c r="N7">
+        <v>1329723.069612419</v>
+      </c>
+      <c r="O7">
+        <v>0</v>
+      </c>
+      <c r="P7">
+        <v>895579.75115197909</v>
+      </c>
+      <c r="Q7">
         <v>0</v>
       </c>
     </row>
@@ -18493,52 +18492,52 @@
       <c r="A8" t="s">
         <v>269</v>
       </c>
-      <c r="B8" s="6">
-        <v>0</v>
-      </c>
-      <c r="C8" s="5">
+      <c r="B8">
+        <v>0</v>
+      </c>
+      <c r="C8">
         <v>-5.0000301997463072</v>
       </c>
-      <c r="D8" s="5">
-        <v>0</v>
-      </c>
-      <c r="E8" s="5">
+      <c r="D8">
+        <v>0</v>
+      </c>
+      <c r="E8">
         <v>4.8749837646976886</v>
       </c>
-      <c r="F8" s="6">
-        <v>0</v>
-      </c>
-      <c r="G8" s="6">
-        <v>0</v>
-      </c>
-      <c r="H8" s="6">
-        <v>0</v>
-      </c>
-      <c r="I8" s="6">
-        <v>0</v>
-      </c>
-      <c r="J8" s="6">
-        <v>0</v>
-      </c>
-      <c r="K8" s="6">
-        <v>0</v>
-      </c>
-      <c r="L8" s="6">
-        <v>0</v>
-      </c>
-      <c r="M8" s="6">
-        <v>0</v>
-      </c>
-      <c r="N8" s="6">
-        <v>0</v>
-      </c>
-      <c r="O8" s="6">
-        <v>0</v>
-      </c>
-      <c r="P8" s="6">
-        <v>0</v>
-      </c>
-      <c r="Q8" s="6">
+      <c r="F8">
+        <v>0</v>
+      </c>
+      <c r="G8">
+        <v>0</v>
+      </c>
+      <c r="H8">
+        <v>0</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+      <c r="J8">
+        <v>0</v>
+      </c>
+      <c r="K8">
+        <v>0</v>
+      </c>
+      <c r="L8">
+        <v>0</v>
+      </c>
+      <c r="M8">
+        <v>0</v>
+      </c>
+      <c r="N8">
+        <v>0</v>
+      </c>
+      <c r="O8">
+        <v>0</v>
+      </c>
+      <c r="P8">
+        <v>0</v>
+      </c>
+      <c r="Q8">
         <v>0</v>
       </c>
     </row>
@@ -18546,52 +18545,52 @@
       <c r="A9" t="s">
         <v>270</v>
       </c>
-      <c r="B9" s="6">
-        <v>130349.249629283</v>
-      </c>
-      <c r="C9" s="5">
-        <v>-6.5166760901829202</v>
-      </c>
-      <c r="D9" s="5">
-        <v>0</v>
-      </c>
-      <c r="E9" s="5">
-        <v>5.0343896711808602</v>
-      </c>
-      <c r="F9" s="6">
-        <v>1836783.8456006399</v>
-      </c>
-      <c r="G9" s="6">
-        <v>972876.63394495798</v>
-      </c>
-      <c r="H9" s="6">
-        <v>972876.63394495798</v>
-      </c>
-      <c r="I9" s="6">
-        <v>0</v>
-      </c>
-      <c r="J9" s="6">
-        <v>0</v>
-      </c>
-      <c r="K9" s="6">
-        <v>0</v>
-      </c>
-      <c r="L9" s="7">
-        <v>5131056.6994807497</v>
-      </c>
-      <c r="M9" s="7">
-        <v>9812139.0623499602</v>
-      </c>
-      <c r="N9" s="7">
-        <v>6517866.20846985</v>
-      </c>
-      <c r="O9" s="6">
-        <v>0</v>
-      </c>
-      <c r="P9" s="7">
-        <v>4186623.0819099899</v>
-      </c>
-      <c r="Q9" s="6">
+      <c r="B9">
+        <v>184419.5</v>
+      </c>
+      <c r="C9">
+        <v>-6.5166760901829237</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9">
+        <v>5.0343896711808611</v>
+      </c>
+      <c r="F9">
+        <v>2598976.1566397501</v>
+      </c>
+      <c r="G9">
+        <v>1370528.006549042</v>
+      </c>
+      <c r="H9">
+        <v>1370528.006549042</v>
+      </c>
+      <c r="I9">
+        <v>0</v>
+      </c>
+      <c r="J9">
+        <v>0</v>
+      </c>
+      <c r="K9">
+        <v>0</v>
+      </c>
+      <c r="L9">
+        <v>7259680.7501828391</v>
+      </c>
+      <c r="M9">
+        <v>13876410.181178899</v>
+      </c>
+      <c r="N9">
+        <v>9215705.5876358133</v>
+      </c>
+      <c r="O9">
+        <v>0</v>
+      </c>
+      <c r="P9">
+        <v>5922635.9457165301</v>
+      </c>
+      <c r="Q9">
         <v>0</v>
       </c>
     </row>
@@ -18599,52 +18598,52 @@
       <c r="A10" t="s">
         <v>271</v>
       </c>
-      <c r="B10" s="6">
-        <v>238490.15752252701</v>
-      </c>
-      <c r="C10" s="5">
-        <v>-6.5166760901829202</v>
-      </c>
-      <c r="D10" s="5">
-        <v>0</v>
-      </c>
-      <c r="E10" s="5">
-        <v>5.0343896711808602</v>
-      </c>
-      <c r="F10" s="6">
-        <v>3360624.39882062</v>
-      </c>
-      <c r="G10" s="6">
-        <v>1779998.7521170501</v>
-      </c>
-      <c r="H10" s="6">
-        <v>1779998.7521170501</v>
-      </c>
-      <c r="I10" s="6">
-        <v>0</v>
-      </c>
-      <c r="J10" s="6">
-        <v>0</v>
-      </c>
-      <c r="K10" s="6">
-        <v>0</v>
-      </c>
-      <c r="L10" s="6">
-        <v>9387906.1367551591</v>
-      </c>
-      <c r="M10" s="7">
-        <v>17952528.282809999</v>
-      </c>
-      <c r="N10" s="7">
-        <v>11925246.544875501</v>
-      </c>
-      <c r="O10" s="6">
-        <v>0</v>
-      </c>
-      <c r="P10" s="7">
-        <v>7659947.4191974998</v>
-      </c>
-      <c r="Q10" s="6">
+      <c r="B10">
+        <v>184419.5</v>
+      </c>
+      <c r="C10">
+        <v>-6.5166760901829237</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10">
+        <v>5.0343896711808611</v>
+      </c>
+      <c r="F10">
+        <v>2598976.1566397501</v>
+      </c>
+      <c r="G10">
+        <v>1370528.006549042</v>
+      </c>
+      <c r="H10">
+        <v>1370528.006549042</v>
+      </c>
+      <c r="I10">
+        <v>0</v>
+      </c>
+      <c r="J10">
+        <v>0</v>
+      </c>
+      <c r="K10">
+        <v>0</v>
+      </c>
+      <c r="L10">
+        <v>7259680.7501828391</v>
+      </c>
+      <c r="M10">
+        <v>13876410.181178899</v>
+      </c>
+      <c r="N10">
+        <v>9215705.5876358133</v>
+      </c>
+      <c r="O10">
+        <v>0</v>
+      </c>
+      <c r="P10">
+        <v>5922635.9457165301</v>
+      </c>
+      <c r="Q10">
         <v>0</v>
       </c>
     </row>
@@ -18652,52 +18651,52 @@
       <c r="A11" t="s">
         <v>272</v>
       </c>
-      <c r="B11" s="6">
+      <c r="B11">
         <v>368839</v>
       </c>
-      <c r="C11" s="5">
+      <c r="C11">
         <v>-6.5166760901829237</v>
       </c>
-      <c r="D11" s="5">
-        <v>0</v>
-      </c>
-      <c r="E11" s="5">
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11">
         <v>5.0343896711808611</v>
       </c>
-      <c r="F11" s="6">
+      <c r="F11">
         <v>5197952.3132795002</v>
       </c>
-      <c r="G11" s="6">
+      <c r="G11">
         <v>2741056.013098083</v>
       </c>
-      <c r="H11" s="6">
+      <c r="H11">
         <v>2741056.013098083</v>
       </c>
-      <c r="I11" s="6">
-        <v>0</v>
-      </c>
-      <c r="J11" s="6">
-        <v>0</v>
-      </c>
-      <c r="K11" s="6">
-        <v>0</v>
-      </c>
-      <c r="L11" s="6">
+      <c r="I11">
+        <v>0</v>
+      </c>
+      <c r="J11">
+        <v>0</v>
+      </c>
+      <c r="K11">
+        <v>0</v>
+      </c>
+      <c r="L11">
         <v>14519361.50036568</v>
       </c>
-      <c r="M11" s="6">
+      <c r="M11">
         <v>27752820.362357799</v>
       </c>
-      <c r="N11" s="6">
+      <c r="N11">
         <v>18431411.17527163</v>
       </c>
-      <c r="O11" s="6">
-        <v>0</v>
-      </c>
-      <c r="P11" s="6">
+      <c r="O11">
+        <v>0</v>
+      </c>
+      <c r="P11">
         <v>11845271.89143306</v>
       </c>
-      <c r="Q11" s="6">
+      <c r="Q11">
         <v>0</v>
       </c>
     </row>
@@ -18705,52 +18704,52 @@
       <c r="A12" t="s">
         <v>273</v>
       </c>
-      <c r="B12" s="6">
+      <c r="B12">
         <v>9381.7774113233681</v>
       </c>
-      <c r="C12" s="5">
+      <c r="C12">
         <v>-6.5166760901829237</v>
       </c>
-      <c r="D12" s="5">
-        <v>0</v>
-      </c>
-      <c r="E12" s="5">
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12">
         <v>5.0343896711808611</v>
       </c>
-      <c r="F12" s="6">
+      <c r="F12">
         <v>148741.82379735971</v>
       </c>
-      <c r="G12" s="6">
+      <c r="G12">
         <v>74370.911898679857</v>
       </c>
-      <c r="H12" s="6">
+      <c r="H12">
         <v>74370.911898679857</v>
       </c>
-      <c r="I12" s="6">
-        <v>0</v>
-      </c>
-      <c r="J12" s="6">
-        <v>0</v>
-      </c>
-      <c r="K12" s="6">
-        <v>0</v>
-      </c>
-      <c r="L12" s="6">
+      <c r="I12">
+        <v>0</v>
+      </c>
+      <c r="J12">
+        <v>0</v>
+      </c>
+      <c r="K12">
+        <v>0</v>
+      </c>
+      <c r="L12">
         <v>385711.12540703168</v>
       </c>
-      <c r="M12" s="6">
+      <c r="M12">
         <v>710569.37732459186</v>
       </c>
-      <c r="N12" s="6">
+      <c r="N12">
         <v>473600.07571491989</v>
       </c>
-      <c r="O12" s="6">
-        <v>0</v>
-      </c>
-      <c r="P12" s="6">
+      <c r="O12">
+        <v>0</v>
+      </c>
+      <c r="P12">
         <v>300061.24755146692</v>
       </c>
-      <c r="Q12" s="6">
+      <c r="Q12">
         <v>0</v>
       </c>
     </row>
@@ -18758,52 +18757,52 @@
       <c r="A13" t="s">
         <v>274</v>
       </c>
-      <c r="B13" s="6">
+      <c r="B13">
         <v>10875.722527829839</v>
       </c>
-      <c r="C13" s="5">
+      <c r="C13">
         <v>-6.044278189882994</v>
       </c>
-      <c r="D13" s="5">
-        <v>0</v>
-      </c>
-      <c r="E13" s="5">
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13">
         <v>4.9847386511287253</v>
       </c>
-      <c r="F13" s="6">
+      <c r="F13">
         <v>12017.673393251969</v>
       </c>
-      <c r="G13" s="6">
+      <c r="G13">
         <v>10005.66472560345</v>
       </c>
-      <c r="H13" s="6">
+      <c r="H13">
         <v>10005.66472560345</v>
       </c>
-      <c r="I13" s="6">
-        <v>0</v>
-      </c>
-      <c r="J13" s="6">
-        <v>0</v>
-      </c>
-      <c r="K13" s="6">
-        <v>0</v>
-      </c>
-      <c r="L13" s="6">
+      <c r="I13">
+        <v>0</v>
+      </c>
+      <c r="J13">
+        <v>0</v>
+      </c>
+      <c r="K13">
+        <v>0</v>
+      </c>
+      <c r="L13">
         <v>282231.50407453772</v>
       </c>
-      <c r="M13" s="6">
+      <c r="M13">
         <v>677567.50018944137</v>
       </c>
-      <c r="N13" s="6">
+      <c r="N13">
         <v>407353.66950815573</v>
       </c>
-      <c r="O13" s="6">
-        <v>0</v>
-      </c>
-      <c r="P13" s="6">
+      <c r="O13">
+        <v>0</v>
+      </c>
+      <c r="P13">
         <v>327467.08392047661</v>
       </c>
-      <c r="Q13" s="6">
+      <c r="Q13">
         <v>0</v>
       </c>
     </row>
@@ -18811,52 +18810,52 @@
       <c r="A14" t="s">
         <v>275</v>
       </c>
-      <c r="B14" s="6">
+      <c r="B14">
         <v>42274.274414881816</v>
       </c>
-      <c r="C14" s="5">
+      <c r="C14">
         <v>-1.2807860584197921</v>
       </c>
-      <c r="D14" s="5">
-        <v>0</v>
-      </c>
-      <c r="E14" s="5">
+      <c r="D14">
+        <v>0</v>
+      </c>
+      <c r="E14">
         <v>2.5860796726634172</v>
       </c>
-      <c r="F14" s="6">
+      <c r="F14">
         <v>549069.84811508202</v>
       </c>
-      <c r="G14" s="6">
+      <c r="G14">
         <v>664478.67296891147</v>
       </c>
-      <c r="H14" s="6">
+      <c r="H14">
         <v>407774.31000719138</v>
       </c>
-      <c r="I14" s="6">
-        <v>0</v>
-      </c>
-      <c r="J14" s="6">
+      <c r="I14">
+        <v>0</v>
+      </c>
+      <c r="J14">
         <v>176991.48534691479</v>
       </c>
-      <c r="K14" s="6">
-        <v>0</v>
-      </c>
-      <c r="L14" s="6">
+      <c r="K14">
+        <v>0</v>
+      </c>
+      <c r="L14">
         <v>831792.08184248838</v>
       </c>
-      <c r="M14" s="6">
+      <c r="M14">
         <v>1016548.172944742</v>
       </c>
-      <c r="N14" s="6">
+      <c r="N14">
         <v>477121.57625561551</v>
       </c>
-      <c r="O14" s="6">
-        <v>0</v>
-      </c>
-      <c r="P14" s="6">
+      <c r="O14">
+        <v>0</v>
+      </c>
+      <c r="P14">
         <v>317012.96233042493</v>
       </c>
-      <c r="Q14" s="6">
+      <c r="Q14">
         <v>0</v>
       </c>
     </row>
@@ -18864,52 +18863,52 @@
       <c r="A15" t="s">
         <v>276</v>
       </c>
-      <c r="B15" s="6">
+      <c r="B15">
         <v>48672</v>
       </c>
-      <c r="C15" s="5">
-        <v>0</v>
-      </c>
-      <c r="D15" s="5">
-        <v>0</v>
-      </c>
-      <c r="E15" s="5">
-        <v>0</v>
-      </c>
-      <c r="F15" s="6">
+      <c r="C15">
+        <v>0</v>
+      </c>
+      <c r="D15">
+        <v>0</v>
+      </c>
+      <c r="E15">
+        <v>0</v>
+      </c>
+      <c r="F15">
         <v>685470.48959999997</v>
       </c>
-      <c r="G15" s="6">
+      <c r="G15">
         <v>685470.48959999997</v>
       </c>
-      <c r="H15" s="6">
+      <c r="H15">
         <v>1370928</v>
       </c>
-      <c r="I15" s="6">
-        <v>0</v>
-      </c>
-      <c r="J15" s="6">
-        <v>0</v>
-      </c>
-      <c r="K15" s="6">
-        <v>0</v>
-      </c>
-      <c r="L15" s="6">
+      <c r="I15">
+        <v>0</v>
+      </c>
+      <c r="J15">
+        <v>0</v>
+      </c>
+      <c r="K15">
+        <v>0</v>
+      </c>
+      <c r="L15">
         <v>685470.48959999997</v>
       </c>
-      <c r="M15" s="6">
+      <c r="M15">
         <v>685470.48959999997</v>
       </c>
-      <c r="N15" s="6">
+      <c r="N15">
         <v>1370928</v>
       </c>
-      <c r="O15" s="6">
-        <v>0</v>
-      </c>
-      <c r="P15" s="6">
-        <v>0</v>
-      </c>
-      <c r="Q15" s="6">
+      <c r="O15">
+        <v>0</v>
+      </c>
+      <c r="P15">
+        <v>0</v>
+      </c>
+      <c r="Q15">
         <v>0</v>
       </c>
     </row>
@@ -18917,52 +18916,52 @@
       <c r="A16" t="s">
         <v>277</v>
       </c>
-      <c r="B16" s="6">
+      <c r="B16">
         <v>20555.95319345692</v>
       </c>
-      <c r="C16" s="5">
+      <c r="C16">
         <v>-0.25000150998731557</v>
       </c>
-      <c r="D16" s="5">
-        <v>0</v>
-      </c>
-      <c r="E16" s="5">
+      <c r="D16">
+        <v>0</v>
+      </c>
+      <c r="E16">
         <v>5.839900000000001</v>
       </c>
-      <c r="F16" s="6">
+      <c r="F16">
         <v>1599.22575051335</v>
       </c>
-      <c r="G16" s="6">
+      <c r="G16">
         <v>1175.7890949070379</v>
       </c>
-      <c r="H16" s="6">
+      <c r="H16">
         <v>1175.7890949070379</v>
       </c>
-      <c r="I16" s="6">
-        <v>0</v>
-      </c>
-      <c r="J16" s="6">
-        <v>0</v>
-      </c>
-      <c r="K16" s="6">
-        <v>0</v>
-      </c>
-      <c r="L16" s="6">
+      <c r="I16">
+        <v>0</v>
+      </c>
+      <c r="J16">
+        <v>0</v>
+      </c>
+      <c r="K16">
+        <v>0</v>
+      </c>
+      <c r="L16">
         <v>702648.33383750753</v>
       </c>
-      <c r="M16" s="6">
+      <c r="M16">
         <v>703509.65977615339</v>
       </c>
-      <c r="N16" s="6">
+      <c r="N16">
         <v>2460.5516891592529</v>
       </c>
-      <c r="O16" s="6">
-        <v>0</v>
-      </c>
-      <c r="P16" s="6">
+      <c r="O16">
+        <v>0</v>
+      </c>
+      <c r="P16">
         <v>30011.359029608269</v>
       </c>
-      <c r="Q16" s="6">
+      <c r="Q16">
         <v>0</v>
       </c>
     </row>
@@ -18970,52 +18969,52 @@
       <c r="A17" t="s">
         <v>278</v>
       </c>
-      <c r="B17" s="6">
+      <c r="B17">
         <v>30635</v>
       </c>
-      <c r="C17" s="5">
-        <v>0</v>
-      </c>
-      <c r="D17" s="5">
+      <c r="C17">
+        <v>0</v>
+      </c>
+      <c r="D17">
         <v>-5.0601298473999998</v>
       </c>
-      <c r="E17" s="5">
+      <c r="E17">
         <v>1.8101298474</v>
       </c>
-      <c r="F17" s="6">
+      <c r="F17">
         <v>66918.482616250083</v>
       </c>
-      <c r="G17" s="6">
+      <c r="G17">
         <v>66918.482616250083</v>
       </c>
-      <c r="H17" s="6">
+      <c r="H17">
         <v>66918.482616250083</v>
       </c>
-      <c r="I17" s="6">
-        <v>0</v>
-      </c>
-      <c r="J17" s="6">
-        <v>0</v>
-      </c>
-      <c r="K17" s="6">
-        <v>0</v>
-      </c>
-      <c r="L17" s="6">
+      <c r="I17">
+        <v>0</v>
+      </c>
+      <c r="J17">
+        <v>0</v>
+      </c>
+      <c r="K17">
+        <v>0</v>
+      </c>
+      <c r="L17">
         <v>951702.74915314373</v>
       </c>
-      <c r="M17" s="6">
+      <c r="M17">
         <v>167296.20654062519</v>
       </c>
-      <c r="N17" s="6">
+      <c r="N17">
         <v>851325.0252287687</v>
       </c>
-      <c r="O17" s="6">
-        <v>0</v>
-      </c>
-      <c r="P17" s="6">
-        <v>0</v>
-      </c>
-      <c r="Q17" s="6">
+      <c r="O17">
+        <v>0</v>
+      </c>
+      <c r="P17">
+        <v>0</v>
+      </c>
+      <c r="Q17">
         <v>280601.03951844678</v>
       </c>
     </row>
@@ -19023,52 +19022,52 @@
       <c r="A18" t="s">
         <v>279</v>
       </c>
-      <c r="B18" s="6">
+      <c r="B18">
         <v>11983.85</v>
       </c>
-      <c r="C18" s="5">
-        <v>0</v>
-      </c>
-      <c r="D18" s="5">
+      <c r="C18">
+        <v>0</v>
+      </c>
+      <c r="D18">
         <v>5.0601298473999998</v>
       </c>
-      <c r="E18" s="5">
+      <c r="E18">
         <v>1.8101298474</v>
       </c>
-      <c r="F18" s="6">
+      <c r="F18">
         <v>26177.282777892891</v>
       </c>
-      <c r="G18" s="6">
+      <c r="G18">
         <v>26177.282777892891</v>
       </c>
-      <c r="H18" s="6">
+      <c r="H18">
         <v>26177.282777892891</v>
       </c>
-      <c r="I18" s="6">
-        <v>0</v>
-      </c>
-      <c r="J18" s="6">
-        <v>0</v>
-      </c>
-      <c r="K18" s="6">
-        <v>0</v>
-      </c>
-      <c r="L18" s="6">
+      <c r="I18">
+        <v>0</v>
+      </c>
+      <c r="J18">
+        <v>0</v>
+      </c>
+      <c r="K18">
+        <v>0</v>
+      </c>
+      <c r="L18">
         <v>372288.65645304072</v>
       </c>
-      <c r="M18" s="6">
+      <c r="M18">
         <v>65443.206944732206</v>
       </c>
-      <c r="N18" s="6">
+      <c r="N18">
         <v>333022.73228620138</v>
       </c>
-      <c r="O18" s="6">
-        <v>0</v>
-      </c>
-      <c r="P18" s="6">
-        <v>0</v>
-      </c>
-      <c r="Q18" s="6">
+      <c r="O18">
+        <v>0</v>
+      </c>
+      <c r="P18">
+        <v>0</v>
+      </c>
+      <c r="Q18">
         <v>-109765.9790250739</v>
       </c>
     </row>
@@ -19076,105 +19075,105 @@
       <c r="A19" t="s">
         <v>280</v>
       </c>
-      <c r="B19" s="6">
-        <v>644813.26594601222</v>
-      </c>
-      <c r="C19" s="5">
-        <v>-5.1245107925153039</v>
-      </c>
-      <c r="D19" s="5">
-        <v>-0.14636367734288569</v>
-      </c>
-      <c r="E19" s="5">
-        <v>4.3141657111563703</v>
-      </c>
-      <c r="F19" s="6">
-        <v>9472954.7400160171</v>
-      </c>
-      <c r="G19" s="6">
-        <v>10596987.68614725</v>
-      </c>
-      <c r="H19" s="6">
-        <v>10521957.30151153</v>
-      </c>
-      <c r="I19" s="6">
-        <v>483637.18906450341</v>
-      </c>
-      <c r="J19" s="6">
-        <v>2197421.5800634511</v>
-      </c>
-      <c r="K19" s="6">
-        <v>-236323.9956939207</v>
-      </c>
-      <c r="L19" s="6">
-        <v>21488049.271249719</v>
-      </c>
-      <c r="M19" s="6">
-        <v>39531459.073413692</v>
-      </c>
-      <c r="N19" s="6">
-        <v>27468960.957587171</v>
-      </c>
-      <c r="O19" s="6">
-        <v>0</v>
-      </c>
-      <c r="P19" s="6">
-        <v>16452946.00784969</v>
-      </c>
-      <c r="Q19" s="6">
-        <v>170835.0604933729</v>
+      <c r="B19">
+        <v>643483.91676964494</v>
+      </c>
+      <c r="C19">
+        <v>-5.1194261344784406</v>
+      </c>
+      <c r="D19">
+        <v>-0.1466660445487401</v>
+      </c>
+      <c r="E19">
+        <v>4.3124456905967934</v>
+      </c>
+      <c r="F19">
+        <v>9471040.1355002355</v>
+      </c>
+      <c r="G19">
+        <v>10587510.621740639</v>
+      </c>
+      <c r="H19">
+        <v>10513369.833851829</v>
+      </c>
+      <c r="I19">
+        <v>483157.31306855578</v>
+      </c>
+      <c r="J19">
+        <v>2194742.1092169122</v>
+      </c>
+      <c r="K19">
+        <v>-236161.66489938271</v>
+      </c>
+      <c r="L19">
+        <v>21451873.340650581</v>
+      </c>
+      <c r="M19">
+        <v>39419265.53205514</v>
+      </c>
+      <c r="N19">
+        <v>27391975.412224069</v>
+      </c>
+      <c r="O19">
+        <v>0</v>
+      </c>
+      <c r="P19">
+        <v>16401095.590921391</v>
+      </c>
+      <c r="Q19">
+        <v>170835.06049337299</v>
       </c>
     </row>
     <row r="20" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>281</v>
       </c>
-      <c r="B20" s="6">
+      <c r="B20">
         <v>28187.49375044175</v>
       </c>
-      <c r="C20" s="5">
-        <v>0</v>
-      </c>
-      <c r="D20" s="5">
-        <v>0</v>
-      </c>
-      <c r="E20" s="5">
-        <v>0</v>
-      </c>
-      <c r="F20" s="6">
-        <v>0</v>
-      </c>
-      <c r="G20" s="6">
-        <v>0</v>
-      </c>
-      <c r="H20" s="6">
-        <v>0</v>
-      </c>
-      <c r="I20" s="6">
-        <v>0</v>
-      </c>
-      <c r="J20" s="6">
-        <v>0</v>
-      </c>
-      <c r="K20" s="6">
-        <v>0</v>
-      </c>
-      <c r="L20" s="6">
-        <v>0</v>
-      </c>
-      <c r="M20" s="6">
-        <v>0</v>
-      </c>
-      <c r="N20" s="6">
-        <v>0</v>
-      </c>
-      <c r="O20" s="6">
-        <v>0</v>
-      </c>
-      <c r="P20" s="6">
-        <v>0</v>
-      </c>
-      <c r="Q20" s="6">
+      <c r="C20">
+        <v>0</v>
+      </c>
+      <c r="D20">
+        <v>0</v>
+      </c>
+      <c r="E20">
+        <v>0</v>
+      </c>
+      <c r="F20">
+        <v>0</v>
+      </c>
+      <c r="G20">
+        <v>0</v>
+      </c>
+      <c r="H20">
+        <v>0</v>
+      </c>
+      <c r="I20">
+        <v>0</v>
+      </c>
+      <c r="J20">
+        <v>0</v>
+      </c>
+      <c r="K20">
+        <v>0</v>
+      </c>
+      <c r="L20">
+        <v>0</v>
+      </c>
+      <c r="M20">
+        <v>0</v>
+      </c>
+      <c r="N20">
+        <v>0</v>
+      </c>
+      <c r="O20">
+        <v>0</v>
+      </c>
+      <c r="P20">
+        <v>0</v>
+      </c>
+      <c r="Q20">
         <v>0</v>
       </c>
     </row>
@@ -19182,105 +19181,105 @@
       <c r="A21" t="s">
         <v>282</v>
       </c>
-      <c r="B21" s="6">
-        <v>673000.75969645393</v>
-      </c>
-      <c r="C21" s="5">
-        <v>-4.9098793617822292</v>
-      </c>
-      <c r="D21" s="5">
-        <v>-0.14023348331122509</v>
-      </c>
-      <c r="E21" s="5">
-        <v>4.1334742078117994</v>
-      </c>
-      <c r="F21" s="6">
-        <v>9955109.5568578355</v>
-      </c>
-      <c r="G21" s="6">
-        <v>11758101.70950149</v>
-      </c>
-      <c r="H21" s="6">
-        <v>11202025.14638547</v>
-      </c>
-      <c r="I21" s="6">
-        <v>464229.26849383238</v>
-      </c>
-      <c r="J21" s="6">
-        <v>2769482.811175345</v>
-      </c>
-      <c r="K21" s="6">
-        <v>-219985.07304531839</v>
-      </c>
-      <c r="L21" s="6">
-        <v>21466972.260889929</v>
-      </c>
-      <c r="M21" s="6">
-        <v>39480701.906951189</v>
-      </c>
-      <c r="N21" s="6">
-        <v>27439232.338249389</v>
-      </c>
-      <c r="O21" s="6">
-        <v>848.40165158855962</v>
-      </c>
-      <c r="P21" s="6">
-        <v>16427938.81083866</v>
-      </c>
-      <c r="Q21" s="6">
-        <v>170120.81761970819</v>
+      <c r="B21">
+        <v>671671.41052008665</v>
+      </c>
+      <c r="C21">
+        <v>-4.9045832962821239</v>
+      </c>
+      <c r="D21">
+        <v>-0.1405110286445817</v>
+      </c>
+      <c r="E21">
+        <v>4.1314687515028794</v>
+      </c>
+      <c r="F21">
+        <v>9952729.9414911009</v>
+      </c>
+      <c r="G21">
+        <v>11746692.307297811</v>
+      </c>
+      <c r="H21">
+        <v>11191974.744480871</v>
+      </c>
+      <c r="I21">
+        <v>463731.95688422862</v>
+      </c>
+      <c r="J21">
+        <v>2765909.0335254958</v>
+      </c>
+      <c r="K21">
+        <v>-219798.34772966561</v>
+      </c>
+      <c r="L21">
+        <v>21430773.157658938</v>
+      </c>
+      <c r="M21">
+        <v>39368488.153373629</v>
+      </c>
+      <c r="N21">
+        <v>27362249.460760672</v>
+      </c>
+      <c r="O21">
+        <v>850.91809099842794</v>
+      </c>
+      <c r="P21">
+        <v>16376075.907150229</v>
+      </c>
+      <c r="Q21">
+        <v>170118.2735023734</v>
       </c>
     </row>
     <row r="22" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>283</v>
       </c>
-      <c r="B22" s="6">
+      <c r="B22">
         <v>203762.89798054329</v>
       </c>
-      <c r="C22" s="5">
-        <v>-11.420282641214079</v>
-      </c>
-      <c r="D22" s="5">
-        <v>0</v>
-      </c>
-      <c r="E22" s="5">
-        <v>5.5497794877707518</v>
-      </c>
-      <c r="F22" s="6">
+      <c r="C22">
+        <v>-13.61998050668908</v>
+      </c>
+      <c r="D22">
+        <v>0</v>
+      </c>
+      <c r="E22">
+        <v>5.7809770497370421</v>
+      </c>
+      <c r="F22">
         <v>348952878.90076488</v>
       </c>
-      <c r="G22" s="6">
+      <c r="G22">
         <v>174476439.45038241</v>
       </c>
-      <c r="H22" s="6">
+      <c r="H22">
         <v>174476439.45038241</v>
       </c>
-      <c r="I22" s="6">
-        <v>0</v>
-      </c>
-      <c r="J22" s="6">
-        <v>0</v>
-      </c>
-      <c r="K22" s="6">
-        <v>0</v>
-      </c>
-      <c r="L22" s="6">
-        <v>353322422.41947103</v>
-      </c>
-      <c r="M22" s="6">
-        <v>207327686.3988122</v>
-      </c>
-      <c r="N22" s="6">
-        <v>202958142.88010591</v>
-      </c>
-      <c r="O22" s="6">
-        <v>0</v>
-      </c>
-      <c r="P22" s="6">
-        <v>-5223343.0341883227</v>
-      </c>
-      <c r="Q22" s="6">
+      <c r="I22">
+        <v>0</v>
+      </c>
+      <c r="J22">
+        <v>0</v>
+      </c>
+      <c r="K22">
+        <v>0</v>
+      </c>
+      <c r="L22">
+        <v>353856208.5272454</v>
+      </c>
+      <c r="M22">
+        <v>219084939.4201408</v>
+      </c>
+      <c r="N22">
+        <v>214181609.79366019</v>
+      </c>
+      <c r="O22">
+        <v>0</v>
+      </c>
+      <c r="P22">
+        <v>-2094208.2957158049</v>
+      </c>
+      <c r="Q22">
         <v>0</v>
       </c>
     </row>
@@ -19288,52 +19287,52 @@
       <c r="A23" t="s">
         <v>284</v>
       </c>
-      <c r="B23" s="6">
-        <v>69006.036596403326</v>
-      </c>
-      <c r="C23" s="5">
-        <v>-11.420282641214079</v>
-      </c>
-      <c r="D23" s="5">
-        <v>0</v>
-      </c>
-      <c r="E23" s="5">
-        <v>5.5497794877707518</v>
-      </c>
-      <c r="F23" s="6">
-        <v>967788.48302954319</v>
-      </c>
-      <c r="G23" s="6">
-        <v>617257.07610674994</v>
-      </c>
-      <c r="H23" s="6">
-        <v>617257.07610674994</v>
-      </c>
-      <c r="I23" s="6">
-        <v>0</v>
-      </c>
-      <c r="J23" s="6">
-        <v>0</v>
-      </c>
-      <c r="K23" s="6">
-        <v>0</v>
-      </c>
-      <c r="L23" s="6">
-        <v>3089348.0474239378</v>
-      </c>
-      <c r="M23" s="6">
-        <v>11742610.963531779</v>
-      </c>
-      <c r="N23" s="6">
-        <v>9621051.3991373889</v>
-      </c>
-      <c r="O23" s="6">
-        <v>0</v>
-      </c>
-      <c r="P23" s="6">
-        <v>4337166.2849609861</v>
-      </c>
-      <c r="Q23" s="6">
+      <c r="B23">
+        <v>68415.010008417899</v>
+      </c>
+      <c r="C23">
+        <v>-11.42076496383466</v>
+      </c>
+      <c r="D23">
+        <v>0</v>
+      </c>
+      <c r="E23">
+        <v>5.5498301819209397</v>
+      </c>
+      <c r="F23">
+        <v>951937.32843975385</v>
+      </c>
+      <c r="G23">
+        <v>615866.15912053839</v>
+      </c>
+      <c r="H23">
+        <v>615866.15912053839</v>
+      </c>
+      <c r="I23">
+        <v>0</v>
+      </c>
+      <c r="J23">
+        <v>0</v>
+      </c>
+      <c r="K23">
+        <v>0</v>
+      </c>
+      <c r="L23">
+        <v>3055489.734538178</v>
+      </c>
+      <c r="M23">
+        <v>11646725.228794049</v>
+      </c>
+      <c r="N23">
+        <v>9543172.8226956241</v>
+      </c>
+      <c r="O23">
+        <v>0</v>
+      </c>
+      <c r="P23">
+        <v>4301432.9584629126</v>
+      </c>
+      <c r="Q23">
         <v>0</v>
       </c>
     </row>
@@ -19341,54 +19340,57 @@
       <c r="A24" t="s">
         <v>285</v>
       </c>
-      <c r="B24" s="6">
-        <v>945769.69427340059</v>
-      </c>
-      <c r="C24" s="5">
-        <v>-7.3209600058004138</v>
-      </c>
-      <c r="D24" s="5">
-        <v>-9.9788818963839829E-2</v>
-      </c>
-      <c r="E24" s="5">
-        <v>4.5980146245874653</v>
-      </c>
-      <c r="F24" s="6">
-        <v>499865525.61414582</v>
-      </c>
-      <c r="G24" s="6">
-        <v>342629218.42514449</v>
-      </c>
-      <c r="H24" s="6">
-        <v>343480100.46718019</v>
-      </c>
-      <c r="I24" s="6">
-        <v>691780.40703059547</v>
-      </c>
-      <c r="J24" s="6">
-        <v>-12757977.77672961</v>
-      </c>
-      <c r="K24" s="6">
-        <v>-263827.11582223681</v>
-      </c>
-      <c r="L24" s="6">
-        <v>378481085.78667837</v>
-      </c>
-      <c r="M24" s="6">
-        <v>271925264.04825127</v>
-      </c>
-      <c r="N24" s="6">
-        <v>252790348.33755529</v>
-      </c>
-      <c r="O24" s="6">
-        <v>848.40165158855962</v>
-      </c>
-      <c r="P24" s="6">
-        <v>19078409.288633171</v>
-      </c>
-      <c r="Q24" s="6">
-        <v>170120.81761970819</v>
-      </c>
+      <c r="B24">
+        <v>943849.31850904785</v>
+      </c>
+      <c r="C24">
+        <v>-7.2584327753025857</v>
+      </c>
+      <c r="D24">
+        <v>-9.9991851403164203E-2</v>
+      </c>
+      <c r="E24">
+        <v>4.5903828960116364</v>
+      </c>
+      <c r="F24">
+        <v>497693450.60987389</v>
+      </c>
+      <c r="G24">
+        <v>339734012.62119132</v>
+      </c>
+      <c r="H24">
+        <v>340599884.5231806</v>
+      </c>
+      <c r="I24">
+        <v>685881.77598054614</v>
+      </c>
+      <c r="J24">
+        <v>-12864801.34210356</v>
+      </c>
+      <c r="K24">
+        <v>-263109.39845402492</v>
+      </c>
+      <c r="L24">
+        <v>378342471.41944247</v>
+      </c>
+      <c r="M24">
+        <v>270100152.8023085</v>
+      </c>
+      <c r="N24">
+        <v>251087032.07711649</v>
+      </c>
+      <c r="O24">
+        <v>850.91809099842794</v>
+      </c>
+      <c r="P24">
+        <v>18583300.569897339</v>
+      </c>
+      <c r="Q24">
+        <v>170118.2735023734</v>
+      </c>
+    </row>
+    <row r="26" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="B26" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
correct RNA MoI moving from TT to CoM
</commit_message>
<xml_diff>
--- a/Documentation/IEA-15-240-RWT_tabular.xlsx
+++ b/Documentation/IEA-15-240-RWT_tabular.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gbarter/devel/IEA-15-240-RWT/Documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56B8FCBE-3DEE-7548-9339-C2710B655D08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{978A79B8-E3A9-B444-BF46-B12F78D30C80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4800" yWindow="620" windowWidth="33600" windowHeight="19360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1009,7 +1009,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="2"/>
@@ -1017,6 +1017,7 @@
     <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="1" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="1" xfId="1" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Heading 1" xfId="2" builtinId="16"/>
@@ -18150,71 +18151,71 @@
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1100-000000000000}">
-  <dimension ref="A1:Q26"/>
+  <dimension ref="A1:Q24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13.83203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="12.83203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="13" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="12.83203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="14" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="12.83203125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.33203125" style="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="12.83203125" style="5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.33203125" style="5" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="13" style="6" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.6640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13" style="6" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="12.83203125" style="6" bestFit="1" customWidth="1"/>
+    <col min="12" max="14" width="12.6640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.33203125" style="6" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12.83203125" style="6" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="12.33203125" style="6" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="17" x14ac:dyDescent="0.2">
       <c r="A1" s="1"/>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="7" t="s">
         <v>247</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="4" t="s">
         <v>248</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="4" t="s">
         <v>249</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="4" t="s">
         <v>250</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="7" t="s">
         <v>251</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="7" t="s">
         <v>252</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="7" t="s">
         <v>253</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="7" t="s">
         <v>254</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="7" t="s">
         <v>255</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="7" t="s">
         <v>256</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="7" t="s">
         <v>257</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" s="7" t="s">
         <v>258</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" s="7" t="s">
         <v>259</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" s="7" t="s">
         <v>260</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" s="7" t="s">
         <v>261</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" s="7" t="s">
         <v>262</v>
       </c>
     </row>
@@ -18227,52 +18228,52 @@
       <c r="A3" t="s">
         <v>264</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="6">
         <v>48092.001786537301</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="5">
         <v>-7.0885261800196808</v>
       </c>
-      <c r="D3">
-        <v>0</v>
-      </c>
-      <c r="E3">
+      <c r="D3" s="5">
+        <v>0</v>
+      </c>
+      <c r="E3" s="5">
         <v>5.094493537559762</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="6">
         <v>59002.874691857964</v>
       </c>
-      <c r="G3">
+      <c r="G3" s="6">
         <v>29771.954855978249</v>
       </c>
-      <c r="H3">
+      <c r="H3" s="6">
         <v>29771.954855978249</v>
       </c>
-      <c r="I3">
-        <v>0</v>
-      </c>
-      <c r="J3">
-        <v>0</v>
-      </c>
-      <c r="K3">
-        <v>0</v>
-      </c>
-      <c r="L3">
+      <c r="I3" s="6">
+        <v>0</v>
+      </c>
+      <c r="J3" s="6">
+        <v>0</v>
+      </c>
+      <c r="K3" s="6">
+        <v>0</v>
+      </c>
+      <c r="L3" s="6">
         <v>1306856.7851224421</v>
       </c>
-      <c r="M3">
+      <c r="M3" s="6">
         <v>3694433.844065466</v>
       </c>
-      <c r="N3">
+      <c r="N3" s="6">
         <v>2446579.9336348828</v>
       </c>
-      <c r="O3">
-        <v>0</v>
-      </c>
-      <c r="P3">
+      <c r="O3" s="6">
+        <v>0</v>
+      </c>
+      <c r="P3" s="6">
         <v>1733681.3241244019</v>
       </c>
-      <c r="Q3">
+      <c r="Q3" s="6">
         <v>0</v>
       </c>
     </row>
@@ -18280,52 +18281,52 @@
       <c r="A4" t="s">
         <v>265</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="6">
         <v>13479.28387693245</v>
       </c>
-      <c r="C4">
+      <c r="C4" s="5">
         <v>-5.8950999055777533</v>
       </c>
-      <c r="D4">
-        <v>0</v>
-      </c>
-      <c r="E4">
+      <c r="D4" s="5">
+        <v>0</v>
+      </c>
+      <c r="E4" s="5">
         <v>4.9690593816385773</v>
       </c>
-      <c r="F4">
+      <c r="F4" s="6">
         <v>16537.3964065115</v>
       </c>
-      <c r="G4">
+      <c r="G4" s="6">
         <v>8344.5191750634949</v>
       </c>
-      <c r="H4">
+      <c r="H4" s="6">
         <v>8344.5191750634949</v>
       </c>
-      <c r="I4">
-        <v>0</v>
-      </c>
-      <c r="J4">
-        <v>0</v>
-      </c>
-      <c r="K4">
-        <v>0</v>
-      </c>
-      <c r="L4">
+      <c r="I4" s="6">
+        <v>0</v>
+      </c>
+      <c r="J4" s="6">
+        <v>0</v>
+      </c>
+      <c r="K4" s="6">
+        <v>0</v>
+      </c>
+      <c r="L4" s="6">
         <v>349272.30654858239</v>
       </c>
-      <c r="M4">
+      <c r="M4" s="6">
         <v>809603.75452328555</v>
       </c>
-      <c r="N4">
+      <c r="N4" s="6">
         <v>476868.84438121459</v>
       </c>
-      <c r="O4">
-        <v>0</v>
-      </c>
-      <c r="P4">
+      <c r="O4" s="6">
+        <v>0</v>
+      </c>
+      <c r="P4" s="6">
         <v>393998.33316090098</v>
       </c>
-      <c r="Q4">
+      <c r="Q4" s="6">
         <v>0</v>
       </c>
     </row>
@@ -18333,52 +18334,52 @@
       <c r="A5" t="s">
         <v>266</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="6">
         <v>15734.038486973781</v>
       </c>
-      <c r="C5">
+      <c r="C5" s="5">
         <v>-6.9890739904828534</v>
       </c>
-      <c r="D5">
-        <v>0</v>
-      </c>
-      <c r="E5">
+      <c r="D5" s="5">
+        <v>0</v>
+      </c>
+      <c r="E5" s="5">
         <v>5.0840406912329961</v>
       </c>
-      <c r="F5">
+      <c r="F5" s="6">
         <v>33120.151015079799</v>
       </c>
-      <c r="G5">
+      <c r="G5" s="6">
         <v>22906.137697285991</v>
       </c>
-      <c r="H5">
+      <c r="H5" s="6">
         <v>22906.137697285991</v>
       </c>
-      <c r="I5">
-        <v>0</v>
-      </c>
-      <c r="J5">
-        <v>0</v>
-      </c>
-      <c r="K5">
-        <v>0</v>
-      </c>
-      <c r="L5">
+      <c r="I5" s="6">
+        <v>0</v>
+      </c>
+      <c r="J5" s="6">
+        <v>0</v>
+      </c>
+      <c r="K5" s="6">
+        <v>0</v>
+      </c>
+      <c r="L5" s="6">
         <v>439693.63450568088</v>
       </c>
-      <c r="M5">
+      <c r="M5" s="6">
         <v>1198154.2421317161</v>
       </c>
-      <c r="N5">
+      <c r="N5" s="6">
         <v>791580.75864111481</v>
       </c>
-      <c r="O5">
-        <v>0</v>
-      </c>
-      <c r="P5">
+      <c r="O5" s="6">
+        <v>0</v>
+      </c>
+      <c r="P5" s="6">
         <v>558011.63821907982</v>
       </c>
-      <c r="Q5">
+      <c r="Q5" s="6">
         <v>0</v>
       </c>
     </row>
@@ -18386,52 +18387,52 @@
       <c r="A6" t="s">
         <v>267</v>
       </c>
-      <c r="B6">
-        <v>0</v>
-      </c>
-      <c r="C6">
+      <c r="B6" s="6">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5">
         <v>-5.0000301997463072</v>
       </c>
-      <c r="D6">
-        <v>0</v>
-      </c>
-      <c r="E6">
+      <c r="D6" s="5">
+        <v>0</v>
+      </c>
+      <c r="E6" s="5">
         <v>4.8749837646976886</v>
       </c>
-      <c r="F6">
-        <v>0</v>
-      </c>
-      <c r="G6">
-        <v>0</v>
-      </c>
-      <c r="H6">
-        <v>0</v>
-      </c>
-      <c r="I6">
-        <v>0</v>
-      </c>
-      <c r="J6">
-        <v>0</v>
-      </c>
-      <c r="K6">
-        <v>0</v>
-      </c>
-      <c r="L6">
-        <v>0</v>
-      </c>
-      <c r="M6">
-        <v>0</v>
-      </c>
-      <c r="N6">
-        <v>0</v>
-      </c>
-      <c r="O6">
-        <v>0</v>
-      </c>
-      <c r="P6">
-        <v>0</v>
-      </c>
-      <c r="Q6">
+      <c r="F6" s="6">
+        <v>0</v>
+      </c>
+      <c r="G6" s="6">
+        <v>0</v>
+      </c>
+      <c r="H6" s="6">
+        <v>0</v>
+      </c>
+      <c r="I6" s="6">
+        <v>0</v>
+      </c>
+      <c r="J6" s="6">
+        <v>0</v>
+      </c>
+      <c r="K6" s="6">
+        <v>0</v>
+      </c>
+      <c r="L6" s="6">
+        <v>0</v>
+      </c>
+      <c r="M6" s="6">
+        <v>0</v>
+      </c>
+      <c r="N6" s="6">
+        <v>0</v>
+      </c>
+      <c r="O6" s="6">
+        <v>0</v>
+      </c>
+      <c r="P6" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="6">
         <v>0</v>
       </c>
     </row>
@@ -18439,52 +18440,52 @@
       <c r="A7" t="s">
         <v>268</v>
       </c>
-      <c r="B7">
+      <c r="B7" s="6">
         <v>22961.01507170952</v>
       </c>
-      <c r="C7">
+      <c r="C7" s="5">
         <v>-7.585787127703818</v>
       </c>
-      <c r="D7">
-        <v>0</v>
-      </c>
-      <c r="E7">
+      <c r="D7" s="5">
+        <v>0</v>
+      </c>
+      <c r="E7" s="5">
         <v>5.1467577691935888</v>
       </c>
-      <c r="F7">
+      <c r="F7" s="6">
         <v>16718.527696291269</v>
       </c>
-      <c r="G7">
+      <c r="G7" s="6">
         <v>8359.2638481456361</v>
       </c>
-      <c r="H7">
+      <c r="H7" s="6">
         <v>8359.2638481456361</v>
       </c>
-      <c r="I7">
-        <v>0</v>
-      </c>
-      <c r="J7">
-        <v>0</v>
-      </c>
-      <c r="K7">
-        <v>0</v>
-      </c>
-      <c r="L7">
+      <c r="I7" s="6">
+        <v>0</v>
+      </c>
+      <c r="J7" s="6">
+        <v>0</v>
+      </c>
+      <c r="K7" s="6">
+        <v>0</v>
+      </c>
+      <c r="L7" s="6">
         <v>624844.17374045495</v>
       </c>
-      <c r="M7">
+      <c r="M7" s="6">
         <v>1937848.715656582</v>
       </c>
-      <c r="N7">
+      <c r="N7" s="6">
         <v>1329723.069612419</v>
       </c>
-      <c r="O7">
-        <v>0</v>
-      </c>
-      <c r="P7">
+      <c r="O7" s="6">
+        <v>0</v>
+      </c>
+      <c r="P7" s="6">
         <v>895579.75115197909</v>
       </c>
-      <c r="Q7">
+      <c r="Q7" s="6">
         <v>0</v>
       </c>
     </row>
@@ -18492,52 +18493,52 @@
       <c r="A8" t="s">
         <v>269</v>
       </c>
-      <c r="B8">
-        <v>0</v>
-      </c>
-      <c r="C8">
+      <c r="B8" s="6">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5">
         <v>-5.0000301997463072</v>
       </c>
-      <c r="D8">
-        <v>0</v>
-      </c>
-      <c r="E8">
+      <c r="D8" s="5">
+        <v>0</v>
+      </c>
+      <c r="E8" s="5">
         <v>4.8749837646976886</v>
       </c>
-      <c r="F8">
-        <v>0</v>
-      </c>
-      <c r="G8">
-        <v>0</v>
-      </c>
-      <c r="H8">
-        <v>0</v>
-      </c>
-      <c r="I8">
-        <v>0</v>
-      </c>
-      <c r="J8">
-        <v>0</v>
-      </c>
-      <c r="K8">
-        <v>0</v>
-      </c>
-      <c r="L8">
-        <v>0</v>
-      </c>
-      <c r="M8">
-        <v>0</v>
-      </c>
-      <c r="N8">
-        <v>0</v>
-      </c>
-      <c r="O8">
-        <v>0</v>
-      </c>
-      <c r="P8">
-        <v>0</v>
-      </c>
-      <c r="Q8">
+      <c r="F8" s="6">
+        <v>0</v>
+      </c>
+      <c r="G8" s="6">
+        <v>0</v>
+      </c>
+      <c r="H8" s="6">
+        <v>0</v>
+      </c>
+      <c r="I8" s="6">
+        <v>0</v>
+      </c>
+      <c r="J8" s="6">
+        <v>0</v>
+      </c>
+      <c r="K8" s="6">
+        <v>0</v>
+      </c>
+      <c r="L8" s="6">
+        <v>0</v>
+      </c>
+      <c r="M8" s="6">
+        <v>0</v>
+      </c>
+      <c r="N8" s="6">
+        <v>0</v>
+      </c>
+      <c r="O8" s="6">
+        <v>0</v>
+      </c>
+      <c r="P8" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="6">
         <v>0</v>
       </c>
     </row>
@@ -18545,52 +18546,52 @@
       <c r="A9" t="s">
         <v>270</v>
       </c>
-      <c r="B9">
+      <c r="B9" s="6">
         <v>184419.5</v>
       </c>
-      <c r="C9">
+      <c r="C9" s="5">
         <v>-6.5166760901829237</v>
       </c>
-      <c r="D9">
-        <v>0</v>
-      </c>
-      <c r="E9">
+      <c r="D9" s="5">
+        <v>0</v>
+      </c>
+      <c r="E9" s="5">
         <v>5.0343896711808611</v>
       </c>
-      <c r="F9">
+      <c r="F9" s="6">
         <v>2598976.1566397501</v>
       </c>
-      <c r="G9">
+      <c r="G9" s="6">
         <v>1370528.006549042</v>
       </c>
-      <c r="H9">
+      <c r="H9" s="6">
         <v>1370528.006549042</v>
       </c>
-      <c r="I9">
-        <v>0</v>
-      </c>
-      <c r="J9">
-        <v>0</v>
-      </c>
-      <c r="K9">
-        <v>0</v>
-      </c>
-      <c r="L9">
+      <c r="I9" s="6">
+        <v>0</v>
+      </c>
+      <c r="J9" s="6">
+        <v>0</v>
+      </c>
+      <c r="K9" s="6">
+        <v>0</v>
+      </c>
+      <c r="L9" s="6">
         <v>7259680.7501828391</v>
       </c>
-      <c r="M9">
+      <c r="M9" s="6">
         <v>13876410.181178899</v>
       </c>
-      <c r="N9">
+      <c r="N9" s="6">
         <v>9215705.5876358133</v>
       </c>
-      <c r="O9">
-        <v>0</v>
-      </c>
-      <c r="P9">
+      <c r="O9" s="6">
+        <v>0</v>
+      </c>
+      <c r="P9" s="6">
         <v>5922635.9457165301</v>
       </c>
-      <c r="Q9">
+      <c r="Q9" s="6">
         <v>0</v>
       </c>
     </row>
@@ -18598,52 +18599,52 @@
       <c r="A10" t="s">
         <v>271</v>
       </c>
-      <c r="B10">
+      <c r="B10" s="6">
         <v>184419.5</v>
       </c>
-      <c r="C10">
+      <c r="C10" s="5">
         <v>-6.5166760901829237</v>
       </c>
-      <c r="D10">
-        <v>0</v>
-      </c>
-      <c r="E10">
+      <c r="D10" s="5">
+        <v>0</v>
+      </c>
+      <c r="E10" s="5">
         <v>5.0343896711808611</v>
       </c>
-      <c r="F10">
+      <c r="F10" s="6">
         <v>2598976.1566397501</v>
       </c>
-      <c r="G10">
+      <c r="G10" s="6">
         <v>1370528.006549042</v>
       </c>
-      <c r="H10">
+      <c r="H10" s="6">
         <v>1370528.006549042</v>
       </c>
-      <c r="I10">
-        <v>0</v>
-      </c>
-      <c r="J10">
-        <v>0</v>
-      </c>
-      <c r="K10">
-        <v>0</v>
-      </c>
-      <c r="L10">
+      <c r="I10" s="6">
+        <v>0</v>
+      </c>
+      <c r="J10" s="6">
+        <v>0</v>
+      </c>
+      <c r="K10" s="6">
+        <v>0</v>
+      </c>
+      <c r="L10" s="6">
         <v>7259680.7501828391</v>
       </c>
-      <c r="M10">
+      <c r="M10" s="6">
         <v>13876410.181178899</v>
       </c>
-      <c r="N10">
+      <c r="N10" s="6">
         <v>9215705.5876358133</v>
       </c>
-      <c r="O10">
-        <v>0</v>
-      </c>
-      <c r="P10">
+      <c r="O10" s="6">
+        <v>0</v>
+      </c>
+      <c r="P10" s="6">
         <v>5922635.9457165301</v>
       </c>
-      <c r="Q10">
+      <c r="Q10" s="6">
         <v>0</v>
       </c>
     </row>
@@ -18651,52 +18652,52 @@
       <c r="A11" t="s">
         <v>272</v>
       </c>
-      <c r="B11">
+      <c r="B11" s="6">
         <v>368839</v>
       </c>
-      <c r="C11">
+      <c r="C11" s="5">
         <v>-6.5166760901829237</v>
       </c>
-      <c r="D11">
-        <v>0</v>
-      </c>
-      <c r="E11">
+      <c r="D11" s="5">
+        <v>0</v>
+      </c>
+      <c r="E11" s="5">
         <v>5.0343896711808611</v>
       </c>
-      <c r="F11">
+      <c r="F11" s="6">
         <v>5197952.3132795002</v>
       </c>
-      <c r="G11">
+      <c r="G11" s="6">
         <v>2741056.013098083</v>
       </c>
-      <c r="H11">
+      <c r="H11" s="6">
         <v>2741056.013098083</v>
       </c>
-      <c r="I11">
-        <v>0</v>
-      </c>
-      <c r="J11">
-        <v>0</v>
-      </c>
-      <c r="K11">
-        <v>0</v>
-      </c>
-      <c r="L11">
+      <c r="I11" s="6">
+        <v>0</v>
+      </c>
+      <c r="J11" s="6">
+        <v>0</v>
+      </c>
+      <c r="K11" s="6">
+        <v>0</v>
+      </c>
+      <c r="L11" s="6">
         <v>14519361.50036568</v>
       </c>
-      <c r="M11">
+      <c r="M11" s="6">
         <v>27752820.362357799</v>
       </c>
-      <c r="N11">
+      <c r="N11" s="6">
         <v>18431411.17527163</v>
       </c>
-      <c r="O11">
-        <v>0</v>
-      </c>
-      <c r="P11">
+      <c r="O11" s="6">
+        <v>0</v>
+      </c>
+      <c r="P11" s="6">
         <v>11845271.89143306</v>
       </c>
-      <c r="Q11">
+      <c r="Q11" s="6">
         <v>0</v>
       </c>
     </row>
@@ -18704,52 +18705,52 @@
       <c r="A12" t="s">
         <v>273</v>
       </c>
-      <c r="B12">
+      <c r="B12" s="6">
         <v>9381.7774113233681</v>
       </c>
-      <c r="C12">
+      <c r="C12" s="5">
         <v>-6.5166760901829237</v>
       </c>
-      <c r="D12">
-        <v>0</v>
-      </c>
-      <c r="E12">
+      <c r="D12" s="5">
+        <v>0</v>
+      </c>
+      <c r="E12" s="5">
         <v>5.0343896711808611</v>
       </c>
-      <c r="F12">
+      <c r="F12" s="6">
         <v>148741.82379735971</v>
       </c>
-      <c r="G12">
+      <c r="G12" s="6">
         <v>74370.911898679857</v>
       </c>
-      <c r="H12">
+      <c r="H12" s="6">
         <v>74370.911898679857</v>
       </c>
-      <c r="I12">
-        <v>0</v>
-      </c>
-      <c r="J12">
-        <v>0</v>
-      </c>
-      <c r="K12">
-        <v>0</v>
-      </c>
-      <c r="L12">
+      <c r="I12" s="6">
+        <v>0</v>
+      </c>
+      <c r="J12" s="6">
+        <v>0</v>
+      </c>
+      <c r="K12" s="6">
+        <v>0</v>
+      </c>
+      <c r="L12" s="6">
         <v>385711.12540703168</v>
       </c>
-      <c r="M12">
+      <c r="M12" s="6">
         <v>710569.37732459186</v>
       </c>
-      <c r="N12">
+      <c r="N12" s="6">
         <v>473600.07571491989</v>
       </c>
-      <c r="O12">
-        <v>0</v>
-      </c>
-      <c r="P12">
+      <c r="O12" s="6">
+        <v>0</v>
+      </c>
+      <c r="P12" s="6">
         <v>300061.24755146692</v>
       </c>
-      <c r="Q12">
+      <c r="Q12" s="6">
         <v>0</v>
       </c>
     </row>
@@ -18757,52 +18758,52 @@
       <c r="A13" t="s">
         <v>274</v>
       </c>
-      <c r="B13">
+      <c r="B13" s="6">
         <v>10875.722527829839</v>
       </c>
-      <c r="C13">
+      <c r="C13" s="5">
         <v>-6.044278189882994</v>
       </c>
-      <c r="D13">
-        <v>0</v>
-      </c>
-      <c r="E13">
+      <c r="D13" s="5">
+        <v>0</v>
+      </c>
+      <c r="E13" s="5">
         <v>4.9847386511287253</v>
       </c>
-      <c r="F13">
+      <c r="F13" s="6">
         <v>12017.673393251969</v>
       </c>
-      <c r="G13">
+      <c r="G13" s="6">
         <v>10005.66472560345</v>
       </c>
-      <c r="H13">
+      <c r="H13" s="6">
         <v>10005.66472560345</v>
       </c>
-      <c r="I13">
-        <v>0</v>
-      </c>
-      <c r="J13">
-        <v>0</v>
-      </c>
-      <c r="K13">
-        <v>0</v>
-      </c>
-      <c r="L13">
+      <c r="I13" s="6">
+        <v>0</v>
+      </c>
+      <c r="J13" s="6">
+        <v>0</v>
+      </c>
+      <c r="K13" s="6">
+        <v>0</v>
+      </c>
+      <c r="L13" s="6">
         <v>282231.50407453772</v>
       </c>
-      <c r="M13">
+      <c r="M13" s="6">
         <v>677567.50018944137</v>
       </c>
-      <c r="N13">
+      <c r="N13" s="6">
         <v>407353.66950815573</v>
       </c>
-      <c r="O13">
-        <v>0</v>
-      </c>
-      <c r="P13">
+      <c r="O13" s="6">
+        <v>0</v>
+      </c>
+      <c r="P13" s="6">
         <v>327467.08392047661</v>
       </c>
-      <c r="Q13">
+      <c r="Q13" s="6">
         <v>0</v>
       </c>
     </row>
@@ -18810,52 +18811,52 @@
       <c r="A14" t="s">
         <v>275</v>
       </c>
-      <c r="B14">
+      <c r="B14" s="6">
         <v>42274.274414881816</v>
       </c>
-      <c r="C14">
+      <c r="C14" s="5">
         <v>-1.2807860584197921</v>
       </c>
-      <c r="D14">
-        <v>0</v>
-      </c>
-      <c r="E14">
+      <c r="D14" s="5">
+        <v>0</v>
+      </c>
+      <c r="E14" s="5">
         <v>2.5860796726634172</v>
       </c>
-      <c r="F14">
+      <c r="F14" s="6">
         <v>549069.84811508202</v>
       </c>
-      <c r="G14">
+      <c r="G14" s="6">
         <v>664478.67296891147</v>
       </c>
-      <c r="H14">
+      <c r="H14" s="6">
         <v>407774.31000719138</v>
       </c>
-      <c r="I14">
-        <v>0</v>
-      </c>
-      <c r="J14">
+      <c r="I14" s="6">
+        <v>0</v>
+      </c>
+      <c r="J14" s="6">
         <v>176991.48534691479</v>
       </c>
-      <c r="K14">
-        <v>0</v>
-      </c>
-      <c r="L14">
+      <c r="K14" s="6">
+        <v>0</v>
+      </c>
+      <c r="L14" s="6">
         <v>831792.08184248838</v>
       </c>
-      <c r="M14">
+      <c r="M14" s="6">
         <v>1016548.172944742</v>
       </c>
-      <c r="N14">
+      <c r="N14" s="6">
         <v>477121.57625561551</v>
       </c>
-      <c r="O14">
-        <v>0</v>
-      </c>
-      <c r="P14">
+      <c r="O14" s="6">
+        <v>0</v>
+      </c>
+      <c r="P14" s="6">
         <v>317012.96233042493</v>
       </c>
-      <c r="Q14">
+      <c r="Q14" s="6">
         <v>0</v>
       </c>
     </row>
@@ -18863,52 +18864,52 @@
       <c r="A15" t="s">
         <v>276</v>
       </c>
-      <c r="B15">
+      <c r="B15" s="6">
         <v>48672</v>
       </c>
-      <c r="C15">
-        <v>0</v>
-      </c>
-      <c r="D15">
-        <v>0</v>
-      </c>
-      <c r="E15">
-        <v>0</v>
-      </c>
-      <c r="F15">
+      <c r="C15" s="5">
+        <v>0</v>
+      </c>
+      <c r="D15" s="5">
+        <v>0</v>
+      </c>
+      <c r="E15" s="5">
+        <v>0</v>
+      </c>
+      <c r="F15" s="6">
         <v>685470.48959999997</v>
       </c>
-      <c r="G15">
+      <c r="G15" s="6">
         <v>685470.48959999997</v>
       </c>
-      <c r="H15">
+      <c r="H15" s="6">
         <v>1370928</v>
       </c>
-      <c r="I15">
-        <v>0</v>
-      </c>
-      <c r="J15">
-        <v>0</v>
-      </c>
-      <c r="K15">
-        <v>0</v>
-      </c>
-      <c r="L15">
+      <c r="I15" s="6">
+        <v>0</v>
+      </c>
+      <c r="J15" s="6">
+        <v>0</v>
+      </c>
+      <c r="K15" s="6">
+        <v>0</v>
+      </c>
+      <c r="L15" s="6">
         <v>685470.48959999997</v>
       </c>
-      <c r="M15">
+      <c r="M15" s="6">
         <v>685470.48959999997</v>
       </c>
-      <c r="N15">
+      <c r="N15" s="6">
         <v>1370928</v>
       </c>
-      <c r="O15">
-        <v>0</v>
-      </c>
-      <c r="P15">
-        <v>0</v>
-      </c>
-      <c r="Q15">
+      <c r="O15" s="6">
+        <v>0</v>
+      </c>
+      <c r="P15" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="6">
         <v>0</v>
       </c>
     </row>
@@ -18916,52 +18917,52 @@
       <c r="A16" t="s">
         <v>277</v>
       </c>
-      <c r="B16">
+      <c r="B16" s="6">
         <v>20555.95319345692</v>
       </c>
-      <c r="C16">
+      <c r="C16" s="5">
         <v>-0.25000150998731557</v>
       </c>
-      <c r="D16">
-        <v>0</v>
-      </c>
-      <c r="E16">
+      <c r="D16" s="5">
+        <v>0</v>
+      </c>
+      <c r="E16" s="5">
         <v>5.839900000000001</v>
       </c>
-      <c r="F16">
+      <c r="F16" s="6">
         <v>1599.22575051335</v>
       </c>
-      <c r="G16">
+      <c r="G16" s="6">
         <v>1175.7890949070379</v>
       </c>
-      <c r="H16">
+      <c r="H16" s="6">
         <v>1175.7890949070379</v>
       </c>
-      <c r="I16">
-        <v>0</v>
-      </c>
-      <c r="J16">
-        <v>0</v>
-      </c>
-      <c r="K16">
-        <v>0</v>
-      </c>
-      <c r="L16">
+      <c r="I16" s="6">
+        <v>0</v>
+      </c>
+      <c r="J16" s="6">
+        <v>0</v>
+      </c>
+      <c r="K16" s="6">
+        <v>0</v>
+      </c>
+      <c r="L16" s="6">
         <v>702648.33383750753</v>
       </c>
-      <c r="M16">
+      <c r="M16" s="6">
         <v>703509.65977615339</v>
       </c>
-      <c r="N16">
+      <c r="N16" s="6">
         <v>2460.5516891592529</v>
       </c>
-      <c r="O16">
-        <v>0</v>
-      </c>
-      <c r="P16">
+      <c r="O16" s="6">
+        <v>0</v>
+      </c>
+      <c r="P16" s="6">
         <v>30011.359029608269</v>
       </c>
-      <c r="Q16">
+      <c r="Q16" s="6">
         <v>0</v>
       </c>
     </row>
@@ -18969,52 +18970,52 @@
       <c r="A17" t="s">
         <v>278</v>
       </c>
-      <c r="B17">
+      <c r="B17" s="6">
         <v>30635</v>
       </c>
-      <c r="C17">
-        <v>0</v>
-      </c>
-      <c r="D17">
+      <c r="C17" s="5">
+        <v>0</v>
+      </c>
+      <c r="D17" s="5">
         <v>-5.0601298473999998</v>
       </c>
-      <c r="E17">
+      <c r="E17" s="5">
         <v>1.8101298474</v>
       </c>
-      <c r="F17">
+      <c r="F17" s="6">
         <v>66918.482616250083</v>
       </c>
-      <c r="G17">
+      <c r="G17" s="6">
         <v>66918.482616250083</v>
       </c>
-      <c r="H17">
+      <c r="H17" s="6">
         <v>66918.482616250083</v>
       </c>
-      <c r="I17">
-        <v>0</v>
-      </c>
-      <c r="J17">
-        <v>0</v>
-      </c>
-      <c r="K17">
-        <v>0</v>
-      </c>
-      <c r="L17">
+      <c r="I17" s="6">
+        <v>0</v>
+      </c>
+      <c r="J17" s="6">
+        <v>0</v>
+      </c>
+      <c r="K17" s="6">
+        <v>0</v>
+      </c>
+      <c r="L17" s="6">
         <v>951702.74915314373</v>
       </c>
-      <c r="M17">
+      <c r="M17" s="6">
         <v>167296.20654062519</v>
       </c>
-      <c r="N17">
+      <c r="N17" s="6">
         <v>851325.0252287687</v>
       </c>
-      <c r="O17">
-        <v>0</v>
-      </c>
-      <c r="P17">
-        <v>0</v>
-      </c>
-      <c r="Q17">
+      <c r="O17" s="6">
+        <v>0</v>
+      </c>
+      <c r="P17" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q17" s="6">
         <v>280601.03951844678</v>
       </c>
     </row>
@@ -19022,52 +19023,52 @@
       <c r="A18" t="s">
         <v>279</v>
       </c>
-      <c r="B18">
+      <c r="B18" s="6">
         <v>11983.85</v>
       </c>
-      <c r="C18">
-        <v>0</v>
-      </c>
-      <c r="D18">
+      <c r="C18" s="5">
+        <v>0</v>
+      </c>
+      <c r="D18" s="5">
         <v>5.0601298473999998</v>
       </c>
-      <c r="E18">
+      <c r="E18" s="5">
         <v>1.8101298474</v>
       </c>
-      <c r="F18">
+      <c r="F18" s="6">
         <v>26177.282777892891</v>
       </c>
-      <c r="G18">
+      <c r="G18" s="6">
         <v>26177.282777892891</v>
       </c>
-      <c r="H18">
+      <c r="H18" s="6">
         <v>26177.282777892891</v>
       </c>
-      <c r="I18">
-        <v>0</v>
-      </c>
-      <c r="J18">
-        <v>0</v>
-      </c>
-      <c r="K18">
-        <v>0</v>
-      </c>
-      <c r="L18">
+      <c r="I18" s="6">
+        <v>0</v>
+      </c>
+      <c r="J18" s="6">
+        <v>0</v>
+      </c>
+      <c r="K18" s="6">
+        <v>0</v>
+      </c>
+      <c r="L18" s="6">
         <v>372288.65645304072</v>
       </c>
-      <c r="M18">
+      <c r="M18" s="6">
         <v>65443.206944732206</v>
       </c>
-      <c r="N18">
+      <c r="N18" s="6">
         <v>333022.73228620138</v>
       </c>
-      <c r="O18">
-        <v>0</v>
-      </c>
-      <c r="P18">
-        <v>0</v>
-      </c>
-      <c r="Q18">
+      <c r="O18" s="6">
+        <v>0</v>
+      </c>
+      <c r="P18" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q18" s="6">
         <v>-109765.9790250739</v>
       </c>
     </row>
@@ -19075,52 +19076,52 @@
       <c r="A19" t="s">
         <v>280</v>
       </c>
-      <c r="B19">
+      <c r="B19" s="6">
         <v>643483.91676964494</v>
       </c>
-      <c r="C19">
+      <c r="C19" s="5">
         <v>-5.1194261344784406</v>
       </c>
-      <c r="D19">
+      <c r="D19" s="5">
         <v>-0.1466660445487401</v>
       </c>
-      <c r="E19">
+      <c r="E19" s="5">
         <v>4.3124456905967934</v>
       </c>
-      <c r="F19">
+      <c r="F19" s="6">
         <v>9471040.1355002355</v>
       </c>
-      <c r="G19">
+      <c r="G19" s="6">
         <v>10587510.621740639</v>
       </c>
-      <c r="H19">
+      <c r="H19" s="6">
         <v>10513369.833851829</v>
       </c>
-      <c r="I19">
+      <c r="I19" s="6">
         <v>483157.31306855578</v>
       </c>
-      <c r="J19">
+      <c r="J19" s="6">
         <v>2194742.1092169122</v>
       </c>
-      <c r="K19">
+      <c r="K19" s="6">
         <v>-236161.66489938271</v>
       </c>
-      <c r="L19">
+      <c r="L19" s="6">
         <v>21451873.340650581</v>
       </c>
-      <c r="M19">
+      <c r="M19" s="6">
         <v>39419265.53205514</v>
       </c>
-      <c r="N19">
+      <c r="N19" s="6">
         <v>27391975.412224069</v>
       </c>
-      <c r="O19">
-        <v>0</v>
-      </c>
-      <c r="P19">
+      <c r="O19" s="6">
+        <v>0</v>
+      </c>
+      <c r="P19" s="6">
         <v>16401095.590921391</v>
       </c>
-      <c r="Q19">
+      <c r="Q19" s="6">
         <v>170835.06049337299</v>
       </c>
     </row>
@@ -19128,52 +19129,52 @@
       <c r="A20" t="s">
         <v>281</v>
       </c>
-      <c r="B20">
+      <c r="B20" s="6">
         <v>28187.49375044175</v>
       </c>
-      <c r="C20">
-        <v>0</v>
-      </c>
-      <c r="D20">
-        <v>0</v>
-      </c>
-      <c r="E20">
-        <v>0</v>
-      </c>
-      <c r="F20">
-        <v>0</v>
-      </c>
-      <c r="G20">
-        <v>0</v>
-      </c>
-      <c r="H20">
-        <v>0</v>
-      </c>
-      <c r="I20">
-        <v>0</v>
-      </c>
-      <c r="J20">
-        <v>0</v>
-      </c>
-      <c r="K20">
-        <v>0</v>
-      </c>
-      <c r="L20">
-        <v>0</v>
-      </c>
-      <c r="M20">
-        <v>0</v>
-      </c>
-      <c r="N20">
-        <v>0</v>
-      </c>
-      <c r="O20">
-        <v>0</v>
-      </c>
-      <c r="P20">
-        <v>0</v>
-      </c>
-      <c r="Q20">
+      <c r="C20" s="5">
+        <v>0</v>
+      </c>
+      <c r="D20" s="5">
+        <v>0</v>
+      </c>
+      <c r="E20" s="5">
+        <v>0</v>
+      </c>
+      <c r="F20" s="6">
+        <v>0</v>
+      </c>
+      <c r="G20" s="6">
+        <v>0</v>
+      </c>
+      <c r="H20" s="6">
+        <v>0</v>
+      </c>
+      <c r="I20" s="6">
+        <v>0</v>
+      </c>
+      <c r="J20" s="6">
+        <v>0</v>
+      </c>
+      <c r="K20" s="6">
+        <v>0</v>
+      </c>
+      <c r="L20" s="6">
+        <v>0</v>
+      </c>
+      <c r="M20" s="6">
+        <v>0</v>
+      </c>
+      <c r="N20" s="6">
+        <v>0</v>
+      </c>
+      <c r="O20" s="6">
+        <v>0</v>
+      </c>
+      <c r="P20" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q20" s="6">
         <v>0</v>
       </c>
     </row>
@@ -19181,52 +19182,52 @@
       <c r="A21" t="s">
         <v>282</v>
       </c>
-      <c r="B21">
+      <c r="B21" s="6">
         <v>671671.41052008665</v>
       </c>
-      <c r="C21">
+      <c r="C21" s="5">
         <v>-4.9045832962821239</v>
       </c>
-      <c r="D21">
+      <c r="D21" s="5">
         <v>-0.1405110286445817</v>
       </c>
-      <c r="E21">
+      <c r="E21" s="5">
         <v>4.1314687515028794</v>
       </c>
-      <c r="F21">
+      <c r="F21" s="6">
         <v>9952729.9414911009</v>
       </c>
-      <c r="G21">
+      <c r="G21" s="6">
         <v>11746692.307297811</v>
       </c>
-      <c r="H21">
+      <c r="H21" s="6">
         <v>11191974.744480871</v>
       </c>
-      <c r="I21">
+      <c r="I21" s="6">
         <v>463731.95688422862</v>
       </c>
-      <c r="J21">
+      <c r="J21" s="6">
         <v>2765909.0335254958</v>
       </c>
-      <c r="K21">
+      <c r="K21" s="6">
         <v>-219798.34772966561</v>
       </c>
-      <c r="L21">
+      <c r="L21" s="6">
         <v>21430773.157658938</v>
       </c>
-      <c r="M21">
+      <c r="M21" s="6">
         <v>39368488.153373629</v>
       </c>
-      <c r="N21">
+      <c r="N21" s="6">
         <v>27362249.460760672</v>
       </c>
-      <c r="O21">
+      <c r="O21" s="6">
         <v>850.91809099842794</v>
       </c>
-      <c r="P21">
+      <c r="P21" s="6">
         <v>16376075.907150229</v>
       </c>
-      <c r="Q21">
+      <c r="Q21" s="6">
         <v>170118.2735023734</v>
       </c>
     </row>
@@ -19234,52 +19235,52 @@
       <c r="A22" t="s">
         <v>283</v>
       </c>
-      <c r="B22">
+      <c r="B22" s="6">
         <v>203762.89798054329</v>
       </c>
-      <c r="C22">
+      <c r="C22" s="5">
         <v>-13.61998050668908</v>
       </c>
-      <c r="D22">
-        <v>0</v>
-      </c>
-      <c r="E22">
+      <c r="D22" s="5">
+        <v>0</v>
+      </c>
+      <c r="E22" s="5">
         <v>5.7809770497370421</v>
       </c>
-      <c r="F22">
+      <c r="F22" s="6">
         <v>348952878.90076488</v>
       </c>
-      <c r="G22">
+      <c r="G22" s="6">
         <v>174476439.45038241</v>
       </c>
-      <c r="H22">
+      <c r="H22" s="6">
         <v>174476439.45038241</v>
       </c>
-      <c r="I22">
-        <v>0</v>
-      </c>
-      <c r="J22">
-        <v>0</v>
-      </c>
-      <c r="K22">
-        <v>0</v>
-      </c>
-      <c r="L22">
+      <c r="I22" s="6">
+        <v>0</v>
+      </c>
+      <c r="J22" s="6">
+        <v>0</v>
+      </c>
+      <c r="K22" s="6">
+        <v>0</v>
+      </c>
+      <c r="L22" s="6">
         <v>353856208.5272454</v>
       </c>
-      <c r="M22">
+      <c r="M22" s="6">
         <v>219084939.4201408</v>
       </c>
-      <c r="N22">
+      <c r="N22" s="6">
         <v>214181609.79366019</v>
       </c>
-      <c r="O22">
-        <v>0</v>
-      </c>
-      <c r="P22">
+      <c r="O22" s="6">
+        <v>0</v>
+      </c>
+      <c r="P22" s="6">
         <v>-2094208.2957158049</v>
       </c>
-      <c r="Q22">
+      <c r="Q22" s="6">
         <v>0</v>
       </c>
     </row>
@@ -19287,52 +19288,52 @@
       <c r="A23" t="s">
         <v>284</v>
       </c>
-      <c r="B23">
+      <c r="B23" s="6">
         <v>68415.010008417899</v>
       </c>
-      <c r="C23">
+      <c r="C23" s="5">
         <v>-11.42076496383466</v>
       </c>
-      <c r="D23">
-        <v>0</v>
-      </c>
-      <c r="E23">
+      <c r="D23" s="5">
+        <v>0</v>
+      </c>
+      <c r="E23" s="5">
         <v>5.5498301819209397</v>
       </c>
-      <c r="F23">
+      <c r="F23" s="6">
         <v>951937.32843975385</v>
       </c>
-      <c r="G23">
+      <c r="G23" s="6">
         <v>615866.15912053839</v>
       </c>
-      <c r="H23">
+      <c r="H23" s="6">
         <v>615866.15912053839</v>
       </c>
-      <c r="I23">
-        <v>0</v>
-      </c>
-      <c r="J23">
-        <v>0</v>
-      </c>
-      <c r="K23">
-        <v>0</v>
-      </c>
-      <c r="L23">
+      <c r="I23" s="6">
+        <v>0</v>
+      </c>
+      <c r="J23" s="6">
+        <v>0</v>
+      </c>
+      <c r="K23" s="6">
+        <v>0</v>
+      </c>
+      <c r="L23" s="6">
         <v>3055489.734538178</v>
       </c>
-      <c r="M23">
+      <c r="M23" s="6">
         <v>11646725.228794049</v>
       </c>
-      <c r="N23">
+      <c r="N23" s="6">
         <v>9543172.8226956241</v>
       </c>
-      <c r="O23">
-        <v>0</v>
-      </c>
-      <c r="P23">
+      <c r="O23" s="6">
+        <v>0</v>
+      </c>
+      <c r="P23" s="6">
         <v>4301432.9584629126</v>
       </c>
-      <c r="Q23">
+      <c r="Q23" s="6">
         <v>0</v>
       </c>
     </row>
@@ -19340,57 +19341,54 @@
       <c r="A24" t="s">
         <v>285</v>
       </c>
-      <c r="B24">
+      <c r="B24" s="6">
         <v>943849.31850904785</v>
       </c>
-      <c r="C24">
+      <c r="C24" s="5">
         <v>-7.2584327753025857</v>
       </c>
-      <c r="D24">
+      <c r="D24" s="5">
         <v>-9.9991851403164203E-2</v>
       </c>
-      <c r="E24">
+      <c r="E24" s="5">
         <v>4.5903828960116364</v>
       </c>
-      <c r="F24">
-        <v>497693450.60987389</v>
-      </c>
-      <c r="G24">
-        <v>339734012.62119132</v>
-      </c>
-      <c r="H24">
-        <v>340599884.5231806</v>
-      </c>
-      <c r="I24">
-        <v>685881.77598054614</v>
-      </c>
-      <c r="J24">
-        <v>-12864801.34210356</v>
-      </c>
-      <c r="K24">
-        <v>-263109.39845402492</v>
-      </c>
-      <c r="L24">
+      <c r="F24" s="6">
+        <v>258991492.22901121</v>
+      </c>
+      <c r="G24" s="6">
+        <v>200466292.98342571</v>
+      </c>
+      <c r="H24" s="6">
+        <v>161574179.6310524</v>
+      </c>
+      <c r="I24" s="6">
+        <v>-684179.93979854928</v>
+      </c>
+      <c r="J24" s="6">
+        <v>50031402.481898241</v>
+      </c>
+      <c r="K24" s="6">
+        <v>603345.94545877166</v>
+      </c>
+      <c r="L24" s="6">
         <v>378342471.41944247</v>
       </c>
-      <c r="M24">
+      <c r="M24" s="6">
         <v>270100152.8023085</v>
       </c>
-      <c r="N24">
+      <c r="N24" s="6">
         <v>251087032.07711649</v>
       </c>
-      <c r="O24">
+      <c r="O24" s="6">
         <v>850.91809099842794</v>
       </c>
-      <c r="P24">
+      <c r="P24" s="6">
         <v>18583300.569897339</v>
       </c>
-      <c r="Q24">
+      <c r="Q24" s="6">
         <v>170118.2735023734</v>
       </c>
-    </row>
-    <row r="26" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="B26" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
one more fix to RNA MoI hopefully
</commit_message>
<xml_diff>
--- a/Documentation/IEA-15-240-RWT_tabular.xlsx
+++ b/Documentation/IEA-15-240-RWT_tabular.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gbarter/devel/IEA-15-240-RWT/Documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{978A79B8-E3A9-B444-BF46-B12F78D30C80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{652ACA03-DC6E-B749-B656-8E52F1970F90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4800" yWindow="620" windowWidth="33600" windowHeight="19360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15340" yWindow="1960" windowWidth="33600" windowHeight="19360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
@@ -18151,7 +18151,7 @@
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1100-000000000000}">
-  <dimension ref="A1:Q24"/>
+  <dimension ref="A1:Q26"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13.83203125" bestFit="1" customWidth="1"/>
@@ -19354,22 +19354,22 @@
         <v>4.5903828960116364</v>
       </c>
       <c r="F24" s="6">
-        <v>258991492.22901121</v>
+        <v>358444604.88218468</v>
       </c>
       <c r="G24" s="6">
-        <v>200466292.98342571</v>
+        <v>200485166.89350221</v>
       </c>
       <c r="H24" s="6">
-        <v>161574179.6310524</v>
+        <v>201351038.79549149</v>
       </c>
       <c r="I24" s="6">
-        <v>-684179.93979854928</v>
+        <v>685881.77598054614</v>
       </c>
       <c r="J24" s="6">
-        <v>50031402.481898241</v>
+        <v>-12864801.34210356</v>
       </c>
       <c r="K24" s="6">
-        <v>603345.94545877166</v>
+        <v>-263109.39845402492</v>
       </c>
       <c r="L24" s="6">
         <v>378342471.41944247</v>
@@ -19389,6 +19389,9 @@
       <c r="Q24" s="6">
         <v>170118.2735023734</v>
       </c>
+    </row>
+    <row r="26" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="C26" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>